<commit_message>
feat: Enhance address map widget to poll database for geocoded coordinate updates and reload parent form after address modal save.
</commit_message>
<xml_diff>
--- a/Reqtodo/Rvk_req_table.xlsx
+++ b/Reqtodo/Rvk_req_table.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,19 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adity/Documents/GitHub/health19/Reqtodo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{B447DA1C-2180-0C42-B6D9-21692EC39946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF72B220-FA8E-EA43-BEF4-CB59488B501F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rvk_req_table" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="133">
   <si>
     <t>Screen/Functionality</t>
   </si>
@@ -413,12 +425,18 @@
   </si>
   <si>
     <t>Add another icon at the topmost bar near the Notifications for new bookings and future bookings, cancellations, rescheduling with different icons on the left; clicking an item opens the booking and removes it from the notification list</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Create In Admin</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -569,7 +587,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -758,6 +776,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -922,7 +946,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -933,6 +957,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1289,13 +1316,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.33203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="170" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="1"/>
+    <col min="3" max="3" width="10.83203125" style="1"/>
+    <col min="4" max="4" width="16.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20" x14ac:dyDescent="0.25">
@@ -1827,7 +1856,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>41</v>
       </c>
@@ -1838,7 +1867,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>41</v>
       </c>
@@ -1849,7 +1878,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>41</v>
       </c>
@@ -1860,18 +1889,18 @@
         <v>127</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B52" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>42</v>
       </c>
@@ -1882,18 +1911,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="B54" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>42</v>
       </c>
@@ -1901,10 +1930,10 @@
         <v>46</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>47</v>
       </c>
@@ -1915,7 +1944,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>47</v>
       </c>
@@ -1926,18 +1955,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="B58" s="6" t="s">
         <v>51</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>52</v>
       </c>
@@ -1948,7 +1977,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>52</v>
       </c>
@@ -1959,18 +1988,21 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B61" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+      <c r="D61" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>57</v>
       </c>
@@ -1981,7 +2013,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>59</v>
       </c>
@@ -1992,7 +2024,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="20" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" ht="20" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>59</v>
       </c>
@@ -2249,7 +2281,7 @@
       <c r="A87" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B87" s="3" t="s">
+      <c r="B87" s="5" t="s">
         <v>86</v>
       </c>
       <c r="C87" s="1" t="s">

</xml_diff>